<commit_message>
début tp1 plus tard
</commit_message>
<xml_diff>
--- a/template/horaire.xlsx
+++ b/template/horaire.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/bd1/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11108B3E-50CE-184B-9B5F-D08067AE1E18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{044D39FE-B7A1-0C4A-9880-BDD6C8D9099D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{A6EAA84D-6E98-BB4B-8698-E4F48E48897D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="61">
   <si>
     <t xml:space="preserve"> Cours </t>
   </si>
@@ -1052,9 +1052,6 @@
       <c r="E17" t="s">
         <v>35</v>
       </c>
-      <c r="F17" t="s">
-        <v>56</v>
-      </c>
       <c r="G17" t="s">
         <v>9</v>
       </c>
@@ -1105,7 +1102,7 @@
         <v>37</v>
       </c>
       <c r="F19" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="G19" t="s">
         <v>9</v>

</xml_diff>